<commit_message>
Replace TestAsset.output_id with multivalued output_ids
An expected output can now be named by several CURIEs, any one of which
counts as the expected answer. For example, sirolimus is CHEBI:9168 and
PUBCHEM.COMPOUND:5284616; node normalization no longer merges these, so
Translator returns them as separate answers.

This is a breaking change: data still using output_id is rejected by the
Pydantic model, and a single CURIE must be given as a one-item list.

- schema: output_id -> output_ids (multivalued uriorcurie)
- regenerate the datamodels and project artifacts with linkml 1.7.8
- convert the examples, add a two-CURIE sirolimus example, and test the
  Pydantic model's handling of the new slot
- bump version to 0.6.0

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S2yuREtzxTuRqVGp8Q8a6d
</commit_message>
<xml_diff>
--- a/project/excel/translator_testing_model.xlsx
+++ b/project/excel/translator_testing_model.xlsx
@@ -1945,7 +1945,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>output_id</t>
+          <t>output_ids</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>output_id</t>
+          <t>output_ids</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>output_id</t>
+          <t>output_ids</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">

</xml_diff>

<commit_message>
Remove test_env from test cases
A suite is the same in every environment, so test cases no longer say
which one they run in: the TestHarness is told. TestCase and
PathfinderTestCase (and so every test case class) drop test_env, and
data that still has it is rejected. TestRunSession keeps it, since a
record of a run says where it ran.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S2yuREtzxTuRqVGp8Q8a6d
</commit_message>
<xml_diff>
--- a/project/excel/translator_testing_model.xlsx
+++ b/project/excel/translator_testing_model.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,37 +534,32 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>test_env</t>
+          <t>id</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>name</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>description</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>tags</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
-        <is>
-          <t>tags</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="5">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"treats"</formula1>
     </dataValidation>
@@ -579,9 +574,6 @@
     </dataValidation>
     <dataValidation sqref="M2:M1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ars,arax,explanatory,improving,aragorn,bte,unsecret,rtxkg2,icees,cam,spoke,molepro,genetics,textmining,cohd,openpredict,collaboratory,connections"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"dev,ci,test,prod"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -594,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,45 +607,37 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>test_env</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>name</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>description</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>tags</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
-        <is>
-          <t>tags</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"AcceptanceTest,BenchmarkTest,QuantitativeTest,StandardsValidationTest,OneHopTest"</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ars,arax,explanatory,improving,aragorn,bte,unsecret,rtxkg2,icees,cam,spoke,molepro,genetics,textmining,cohd,openpredict,collaboratory,connections"</formula1>
-    </dataValidation>
-    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"dev,ci,test,prod"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -666,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -737,37 +721,32 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>test_env</t>
+          <t>id</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>name</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>description</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>tags</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
-        <is>
-          <t>tags</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="5">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"treats"</formula1>
     </dataValidation>
@@ -782,9 +761,6 @@
     </dataValidation>
     <dataValidation sqref="M2:M1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ars,arax,explanatory,improving,aragorn,bte,unsecret,rtxkg2,icees,cam,spoke,molepro,genetics,textmining,cohd,openpredict,collaboratory,connections"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"dev,ci,test,prod"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -797,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -868,37 +844,32 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>test_env</t>
+          <t>id</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>name</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>description</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>tags</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
-        <is>
-          <t>tags</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="5">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"treats"</formula1>
     </dataValidation>
@@ -913,9 +884,6 @@
     </dataValidation>
     <dataValidation sqref="M2:M1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ars,arax,explanatory,improving,aragorn,bte,unsecret,rtxkg2,icees,cam,spoke,molepro,genetics,textmining,cohd,openpredict,collaboratory,connections"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"dev,ci,test,prod"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -928,7 +896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1009,37 +977,32 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>test_env</t>
+          <t>id</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>name</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>description</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>tags</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
-        <is>
-          <t>tags</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="5">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"treats"</formula1>
     </dataValidation>
@@ -1054,9 +1017,6 @@
     </dataValidation>
     <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ars,arax,explanatory,improving,aragorn,bte,unsecret,rtxkg2,icees,cam,spoke,molepro,genetics,textmining,cohd,openpredict,collaboratory,connections"</formula1>
-    </dataValidation>
-    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"dev,ci,test,prod"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add skip and skip_reason to test assets and test cases
Some tests always fail for a known reason, and should be turned off
until the issue behind them is fixed. skip (default false) and an
optional skip_reason go on TestAsset, PathfinderTestAsset, TestCase and
PathfinderTestCase, and so on every asset and test case class; skipping
a test case skips all of its assets. The Test Harness reports skipped
tests as skipped and can be told to run them anyway.

Both fields are optional, so existing data stays valid. Version 0.7.0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S2yuREtzxTuRqVGp8Q8a6d
</commit_message>
<xml_diff>
--- a/project/excel/translator_testing_model.xlsx
+++ b/project/excel/translator_testing_model.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,25 +534,35 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>skip_reason</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>
@@ -586,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -607,25 +617,35 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>skip_reason</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>
@@ -645,252 +665,6 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:R1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>query_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>test_assets</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>preconditions</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>trapi_template</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>test_case_objective</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>test_case_source</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>test_case_predicate_name</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>test_case_predicate_id</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>test_case_input_id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>qualifiers</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>input_category</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>output_category</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>components</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>tags</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>test_runner_settings</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"treats"</formula1>
-    </dataValidation>
-    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ameliorates,treats,three_hop,drug_treats_rare_disease,drug-to-gene"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"AcceptanceTest,BenchmarkTest,QuantitativeTest,StandardsValidationTest,OneHopTest"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SME,SMURF,GitHubUserFeedback,TACT,BenchMark,TranslatorTeam,TestDataLocation"</formula1>
-    </dataValidation>
-    <dataValidation sqref="M2:M1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ars,arax,explanatory,improving,aragorn,bte,unsecret,rtxkg2,icees,cam,spoke,molepro,genetics,textmining,cohd,openpredict,collaboratory,connections"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:R1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>query_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>test_assets</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>preconditions</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>trapi_template</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>test_case_objective</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>test_case_source</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>test_case_predicate_name</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>test_case_predicate_id</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>test_case_input_id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>qualifiers</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>input_category</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>output_category</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>components</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>tags</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>test_runner_settings</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"treats"</formula1>
-    </dataValidation>
-    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ameliorates,treats,three_hop,drug_treats_rare_disease,drug-to-gene"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"AcceptanceTest,BenchmarkTest,QuantitativeTest,StandardsValidationTest,OneHopTest"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SME,SMURF,GitHubUserFeedback,TACT,BenchMark,TranslatorTeam,TestDataLocation"</formula1>
-    </dataValidation>
-    <dataValidation sqref="M2:M1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ars,arax,explanatory,improving,aragorn,bte,unsecret,rtxkg2,icees,cam,spoke,molepro,genetics,textmining,cohd,openpredict,collaboratory,connections"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -902,6 +676,272 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>query_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>test_assets</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>preconditions</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>trapi_template</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>test_case_objective</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>test_case_source</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>test_case_predicate_name</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>test_case_predicate_id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>test_case_input_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>qualifiers</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>input_category</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>output_category</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>components</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>skip_reason</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>test_runner_settings</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"treats"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ameliorates,treats,three_hop,drug_treats_rare_disease,drug-to-gene"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"AcceptanceTest,BenchmarkTest,QuantitativeTest,StandardsValidationTest,OneHopTest"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SME,SMURF,GitHubUserFeedback,TACT,BenchMark,TranslatorTeam,TestDataLocation"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ars,arax,explanatory,improving,aragorn,bte,unsecret,rtxkg2,icees,cam,spoke,molepro,genetics,textmining,cohd,openpredict,collaboratory,connections"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>query_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>test_assets</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>preconditions</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>trapi_template</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>test_case_objective</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>test_case_source</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>test_case_predicate_name</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>test_case_predicate_id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>test_case_input_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>qualifiers</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>input_category</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>output_category</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>components</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>skip_reason</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>test_runner_settings</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"treats"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ameliorates,treats,three_hop,drug_treats_rare_disease,drug-to-gene"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"AcceptanceTest,BenchmarkTest,QuantitativeTest,StandardsValidationTest,OneHopTest"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SME,SMURF,GitHubUserFeedback,TACT,BenchMark,TranslatorTeam,TestDataLocation"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ars,arax,explanatory,improving,aragorn,bte,unsecret,rtxkg2,icees,cam,spoke,molepro,genetics,textmining,cohd,openpredict,collaboratory,connections"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>test_run_time</t>
         </is>
       </c>
@@ -977,25 +1017,35 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>skip_reason</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>
@@ -1874,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:X1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1965,25 +2015,35 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>skip_reason</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>
@@ -2008,7 +2068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2074,25 +2134,35 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>skip_reason</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>
@@ -2109,7 +2179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AH1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2250,25 +2320,35 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>skip_reason</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>
@@ -2305,7 +2385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:X1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2396,25 +2476,35 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>skip_reason</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>test_runner_settings</t>
         </is>

</xml_diff>